<commit_message>
fixed is_active model in service schemas
</commit_message>
<xml_diff>
--- a/Members details.xlsx
+++ b/Members details.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nandom\youth_church\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17050" windowHeight="4540"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,10 +35,10 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>Nandom Fyamya</t>
+    <t>Usher PORTAL</t>
   </si>
   <si>
-    <t>07019809922</t>
+    <t>08123456789</t>
   </si>
 </sst>
 </file>

</xml_diff>